<commit_message>
Improve program UX, sample water data, and view encoding cues
Turn off the Filters coverage check by default while keeping program
confidence greying, make insights action- or consequence-led per program,
and seed water-cohort sample assets so that goal is not 100% clear. Add
Pack/Iso encoding captions, drop the Iso compass, and ship related drawer
and create-program UI updates.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Enertiv Product Management/25-asset-level-esg-data-NY.xlsx
+++ b/Enertiv Product Management/25-asset-level-esg-data-NY.xlsx
@@ -2535,7 +2535,7 @@
         <v>17444.1</v>
       </c>
       <c r="T2" s="7" t="n">
-        <v>212469</v>
+        <v>1980000</v>
       </c>
       <c r="U2" s="7" t="n">
         <v>19186</v>
@@ -2846,7 +2846,7 @@
         <v>196574.1</v>
       </c>
       <c r="T5" s="7" t="n">
-        <v>2367714</v>
+        <v>3089988</v>
       </c>
       <c r="U5" s="7" t="n">
         <v>0</v>
@@ -2945,7 +2945,7 @@
         <v>123121.8</v>
       </c>
       <c r="T6" s="7" t="n">
-        <v>1886979</v>
+        <v>2757078</v>
       </c>
       <c r="U6" s="7" t="n">
         <v>0</v>
@@ -3143,7 +3143,7 @@
         <v>55564.4</v>
       </c>
       <c r="T8" s="7" t="n">
-        <v>441890</v>
+        <v>1978020</v>
       </c>
       <c r="U8" s="7" t="n">
         <v>48513</v>
@@ -3638,7 +3638,7 @@
         <v>308634.4</v>
       </c>
       <c r="T13" s="7" t="n">
-        <v>3652482</v>
+        <v>4378752</v>
       </c>
       <c r="U13" s="7" t="n">
         <v>65682</v>
@@ -3836,7 +3836,7 @@
         <v>126417.8</v>
       </c>
       <c r="T15" s="7" t="n">
-        <v>2671026</v>
+        <v>5231520</v>
       </c>
       <c r="U15" s="7" t="n">
         <v>265789</v>
@@ -3935,7 +3935,7 @@
         <v>230191.4</v>
       </c>
       <c r="T16" s="7" t="n">
-        <v>2052829</v>
+        <v>3692520</v>
       </c>
       <c r="U16" s="7" t="n">
         <v>102710</v>
@@ -4034,7 +4034,7 @@
         <v>732936.5</v>
       </c>
       <c r="T17" s="7" t="n">
-        <v>5397694</v>
+        <v>6979005</v>
       </c>
       <c r="U17" s="7" t="n">
         <v>289701</v>
@@ -4232,7 +4232,7 @@
         <v>66392</v>
       </c>
       <c r="T19" s="7" t="n">
-        <v>341125</v>
+        <v>796320</v>
       </c>
       <c r="U19" s="7" t="n">
         <v>44876</v>
@@ -4727,7 +4727,7 @@
         <v>375112.6</v>
       </c>
       <c r="T24" s="7" t="n">
-        <v>4022033</v>
+        <v>4651020</v>
       </c>
       <c r="U24" s="7" t="n">
         <v>0</v>
@@ -5024,7 +5024,7 @@
         <v>459453.5</v>
       </c>
       <c r="T27" s="7" t="n">
-        <v>3940905</v>
+        <v>8239104</v>
       </c>
       <c r="U27" s="7" t="n">
         <v>0</v>
@@ -5321,7 +5321,7 @@
         <v>715834.4</v>
       </c>
       <c r="T30" s="7" t="n">
-        <v>4709928</v>
+        <v>6881760</v>
       </c>
       <c r="U30" s="7" t="n">
         <v>271138</v>
@@ -8457,7 +8457,7 @@
       </c>
       <c r="H62" s="23" t="n">
         <f aca="false">'Asset-Level Data'!T2</f>
-        <v>212469</v>
+        <v>1980000</v>
       </c>
       <c r="I62" s="23" t="n">
         <f aca="false">F62*(1-$Q$5)</f>
@@ -8468,15 +8468,15 @@
       </c>
       <c r="K62" s="9" t="n">
         <f aca="false">(F62-H62)/(F62-I62)</f>
-        <v>2.05002948560333</v>
+        <v>-36.3558054</v>
       </c>
       <c r="L62" s="23" t="n">
         <f aca="false">H62-I62</f>
-        <v>-48324.94</v>
+        <v>1719206.06</v>
       </c>
       <c r="M62" s="4" t="str">
         <f aca="false">IF(K62&gt;=1,"Target Met",IF(K62&gt;=0.75,"On Track",IF(K62&gt;=0.4,"At Risk","Off Track")))</f>
-        <v>Target Met</v>
+        <v>Off Track</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8595,7 +8595,7 @@
       </c>
       <c r="H65" s="23" t="n">
         <f aca="false">'Asset-Level Data'!T5</f>
-        <v>2367714</v>
+        <v>3089988</v>
       </c>
       <c r="I65" s="23" t="n">
         <f aca="false">F65*(1-$Q$5)</f>
@@ -8606,15 +8606,15 @@
       </c>
       <c r="K65" s="9" t="n">
         <f aca="false">(F65-H65)/(F65-I65)</f>
-        <v>1.82572417710981</v>
+        <v>0.3489888553</v>
       </c>
       <c r="L65" s="23" t="n">
         <f aca="false">H65-I65</f>
-        <v>-403863.235</v>
+        <v>318410.765</v>
       </c>
       <c r="M65" s="4" t="str">
         <f aca="false">IF(K65&gt;=1,"Target Met",IF(K65&gt;=0.75,"On Track",IF(K65&gt;=0.4,"At Risk","Off Track")))</f>
-        <v>Target Met</v>
+        <v>Off Track</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8641,7 +8641,7 @@
       </c>
       <c r="H66" s="23" t="n">
         <f aca="false">'Asset-Level Data'!T6</f>
-        <v>1886979</v>
+        <v>2757078</v>
       </c>
       <c r="I66" s="23" t="n">
         <f aca="false">F66*(1-$Q$5)</f>
@@ -8652,15 +8652,15 @@
       </c>
       <c r="K66" s="9" t="n">
         <f aca="false">(F66-H66)/(F66-I66)</f>
-        <v>1.09064404354257</v>
+        <v>-1.480498353</v>
       </c>
       <c r="L66" s="23" t="n">
         <f aca="false">H66-I66</f>
-        <v>-30674.8049999997</v>
+        <v>839424.195</v>
       </c>
       <c r="M66" s="4" t="str">
         <f aca="false">IF(K66&gt;=1,"Target Met",IF(K66&gt;=0.75,"On Track",IF(K66&gt;=0.4,"At Risk","Off Track")))</f>
-        <v>Target Met</v>
+        <v>Off Track</v>
       </c>
     </row>
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8733,7 +8733,7 @@
       </c>
       <c r="H68" s="23" t="n">
         <f aca="false">'Asset-Level Data'!T8</f>
-        <v>441890</v>
+        <v>1978020</v>
       </c>
       <c r="I68" s="23" t="n">
         <f aca="false">F68*(1-$Q$5)</f>
@@ -8744,15 +8744,15 @@
       </c>
       <c r="K68" s="9" t="n">
         <f aca="false">(F68-H68)/(F68-I68)</f>
-        <v>0.928257680782316</v>
+        <v>-19.02001496</v>
       </c>
       <c r="L68" s="23" t="n">
         <f aca="false">H68-I68</f>
-        <v>5524.565</v>
+        <v>1541654.565</v>
       </c>
       <c r="M68" s="4" t="str">
         <f aca="false">IF(K68&gt;=1,"Target Met",IF(K68&gt;=0.75,"On Track",IF(K68&gt;=0.4,"At Risk","Off Track")))</f>
-        <v>On Track</v>
+        <v>Off Track</v>
       </c>
     </row>
     <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8963,7 +8963,7 @@
       </c>
       <c r="H73" s="23" t="n">
         <f aca="false">'Asset-Level Data'!T13</f>
-        <v>3652482</v>
+        <v>4378752</v>
       </c>
       <c r="I73" s="23" t="n">
         <f aca="false">F73*(1-$Q$5)</f>
@@ -8974,15 +8974,15 @@
       </c>
       <c r="K73" s="9" t="n">
         <f aca="false">(F73-H73)/(F73-I73)</f>
-        <v>1.30814503263477</v>
+        <v>0.2426412171</v>
       </c>
       <c r="L73" s="23" t="n">
         <f aca="false">H73-I73</f>
-        <v>-210038.19</v>
+        <v>516231.81</v>
       </c>
       <c r="M73" s="4" t="str">
         <f aca="false">IF(K73&gt;=1,"Target Met",IF(K73&gt;=0.75,"On Track",IF(K73&gt;=0.4,"At Risk","Off Track")))</f>
-        <v>Target Met</v>
+        <v>Off Track</v>
       </c>
     </row>
     <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9055,7 +9055,7 @@
       </c>
       <c r="H75" s="23" t="n">
         <f aca="false">'Asset-Level Data'!T15</f>
-        <v>2671026</v>
+        <v>5231520</v>
       </c>
       <c r="I75" s="23" t="n">
         <f aca="false">F75*(1-$Q$5)</f>
@@ -9066,15 +9066,15 @@
       </c>
       <c r="K75" s="9" t="n">
         <f aca="false">(F75-H75)/(F75-I75)</f>
-        <v>1.64776154077873</v>
+        <v>-3.163452001</v>
       </c>
       <c r="L75" s="23" t="n">
         <f aca="false">H75-I75</f>
-        <v>-344734.135</v>
+        <v>2215759.865</v>
       </c>
       <c r="M75" s="4" t="str">
         <f aca="false">IF(K75&gt;=1,"Target Met",IF(K75&gt;=0.75,"On Track",IF(K75&gt;=0.4,"At Risk","Off Track")))</f>
-        <v>Target Met</v>
+        <v>Off Track</v>
       </c>
     </row>
     <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9101,7 +9101,7 @@
       </c>
       <c r="H76" s="23" t="n">
         <f aca="false">'Asset-Level Data'!T16</f>
-        <v>2052829</v>
+        <v>3692520</v>
       </c>
       <c r="I76" s="23" t="n">
         <f aca="false">F76*(1-$Q$5)</f>
@@ -9112,15 +9112,15 @@
       </c>
       <c r="K76" s="9" t="n">
         <f aca="false">(F76-H76)/(F76-I76)</f>
-        <v>1.63130045190964</v>
+        <v>-2.390683193</v>
       </c>
       <c r="L76" s="23" t="n">
         <f aca="false">H76-I76</f>
-        <v>-257369.935</v>
+        <v>1382321.065</v>
       </c>
       <c r="M76" s="4" t="str">
         <f aca="false">IF(K76&gt;=1,"Target Met",IF(K76&gt;=0.75,"On Track",IF(K76&gt;=0.4,"At Risk","Off Track")))</f>
-        <v>Target Met</v>
+        <v>Off Track</v>
       </c>
     </row>
     <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9147,7 +9147,7 @@
       </c>
       <c r="H77" s="23" t="n">
         <f aca="false">'Asset-Level Data'!T17</f>
-        <v>5397694</v>
+        <v>6979005</v>
       </c>
       <c r="I77" s="23" t="n">
         <f aca="false">F77*(1-$Q$5)</f>
@@ -9158,15 +9158,15 @@
       </c>
       <c r="K77" s="9" t="n">
         <f aca="false">(F77-H77)/(F77-I77)</f>
-        <v>1.48610435730673</v>
+        <v>-0.03159563939</v>
       </c>
       <c r="L77" s="23" t="n">
         <f aca="false">H77-I77</f>
-        <v>-506478.335</v>
+        <v>1074832.665</v>
       </c>
       <c r="M77" s="4" t="str">
         <f aca="false">IF(K77&gt;=1,"Target Met",IF(K77&gt;=0.75,"On Track",IF(K77&gt;=0.4,"At Risk","Off Track")))</f>
-        <v>Target Met</v>
+        <v>Off Track</v>
       </c>
     </row>
     <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9239,7 +9239,7 @@
       </c>
       <c r="H79" s="23" t="n">
         <f aca="false">'Asset-Level Data'!T19</f>
-        <v>341125</v>
+        <v>796320</v>
       </c>
       <c r="I79" s="23" t="n">
         <f aca="false">F79*(1-$Q$5)</f>
@@ -9250,15 +9250,15 @@
       </c>
       <c r="K79" s="9" t="n">
         <f aca="false">(F79-H79)/(F79-I79)</f>
-        <v>2.01573470443285</v>
+        <v>-4.190438911</v>
       </c>
       <c r="L79" s="23" t="n">
         <f aca="false">H79-I79</f>
-        <v>-74499.585</v>
+        <v>380695.415</v>
       </c>
       <c r="M79" s="4" t="str">
         <f aca="false">IF(K79&gt;=1,"Target Met",IF(K79&gt;=0.75,"On Track",IF(K79&gt;=0.4,"At Risk","Off Track")))</f>
-        <v>Target Met</v>
+        <v>Off Track</v>
       </c>
     </row>
     <row r="80" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9469,7 +9469,7 @@
       </c>
       <c r="H84" s="23" t="n">
         <f aca="false">'Asset-Level Data'!T24</f>
-        <v>4022033</v>
+        <v>4651020</v>
       </c>
       <c r="I84" s="23" t="n">
         <f aca="false">F84*(1-$Q$5)</f>
@@ -9480,15 +9480,15 @@
       </c>
       <c r="K84" s="9" t="n">
         <f aca="false">(F84-H84)/(F84-I84)</f>
-        <v>1.70686086453071</v>
+        <v>0.9312199456</v>
       </c>
       <c r="L84" s="23" t="n">
         <f aca="false">H84-I84</f>
-        <v>-573211.5</v>
+        <v>55775.5</v>
       </c>
       <c r="M84" s="4" t="str">
         <f aca="false">IF(K84&gt;=1,"Target Met",IF(K84&gt;=0.75,"On Track",IF(K84&gt;=0.4,"At Risk","Off Track")))</f>
-        <v>Target Met</v>
+        <v>On Track</v>
       </c>
     </row>
     <row r="85" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9607,7 +9607,7 @@
       </c>
       <c r="H87" s="23" t="n">
         <f aca="false">'Asset-Level Data'!T27</f>
-        <v>3940905</v>
+        <v>8239104</v>
       </c>
       <c r="I87" s="23" t="n">
         <f aca="false">F87*(1-$Q$5)</f>
@@ -9618,15 +9618,15 @@
       </c>
       <c r="K87" s="9" t="n">
         <f aca="false">(F87-H87)/(F87-I87)</f>
-        <v>1.15914574264868</v>
+        <v>-4.847703174</v>
       </c>
       <c r="L87" s="23" t="n">
         <f aca="false">H87-I87</f>
-        <v>-113876.69</v>
+        <v>4184322.31</v>
       </c>
       <c r="M87" s="4" t="str">
         <f aca="false">IF(K87&gt;=1,"Target Met",IF(K87&gt;=0.75,"On Track",IF(K87&gt;=0.4,"At Risk","Off Track")))</f>
-        <v>Target Met</v>
+        <v>Off Track</v>
       </c>
     </row>
     <row r="88" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9745,7 +9745,7 @@
       </c>
       <c r="H90" s="23" t="n">
         <f aca="false">'Asset-Level Data'!T30</f>
-        <v>4709928</v>
+        <v>6881760</v>
       </c>
       <c r="I90" s="23" t="n">
         <f aca="false">F90*(1-$Q$5)</f>
@@ -9756,15 +9756,15 @@
       </c>
       <c r="K90" s="9" t="n">
         <f aca="false">(F90-H90)/(F90-I90)</f>
-        <v>1.92768665775574</v>
+        <v>-0.2575417429</v>
       </c>
       <c r="L90" s="23" t="n">
         <f aca="false">H90-I90</f>
-        <v>-921999.534999999</v>
+        <v>1249832.465</v>
       </c>
       <c r="M90" s="4" t="str">
         <f aca="false">IF(K90&gt;=1,"Target Met",IF(K90&gt;=0.75,"On Track",IF(K90&gt;=0.4,"At Risk","Off Track")))</f>
-        <v>Target Met</v>
+        <v>Off Track</v>
       </c>
     </row>
     <row r="91" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>